<commit_message>
Add external workbook support and weekly schedules
</commit_message>
<xml_diff>
--- a/templates/Sports-template.xlsx
+++ b/templates/Sports-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy" sheetId="1" r:id="Ra120d42a9cd544df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training log" sheetId="2" r:id="Rc96c6f1dce8c4891"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy" sheetId="1" r:id="Rf80fbfa5de234fdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training log" sheetId="2" r:id="R2004f5cabf214ce2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,9 +14,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
-    <x:numFmt numFmtId="200" formatCode="[=1]&quot;TRUE&quot;;[=0]&quot;FALSE&quot;;General"/>
-    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
+  <x:numFmts count="4">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
+    <x:numFmt numFmtId="202" formatCode="[=1]&quot;TRUE&quot;;[=0]&quot;FALSE&quot;;General"/>
+    <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -81,7 +83,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -92,6 +94,8 @@
       <x:alignment horizontal="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:extLst>
         <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -125,7 +129,7 @@
         </x:ext>
       </x:extLst>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
       <x:extLst>
         <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -136,13 +140,19 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -151,7 +161,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="202" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
       <x:extLst>
         <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -165,7 +175,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="203" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -390,6 +400,8 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="38" hidden="0" customWidth="1"/>
     <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="36" hidden="0" customWidth="1"/>
@@ -397,274 +409,435 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="15" t="str">
+      <x:c r="A1" s="17" t="str">
         <x:v>Plan</x:v>
       </x:c>
-      <x:c r="B1" s="15"/>
-      <x:c r="C1" s="15"/>
-      <x:c r="D1" s="15"/>
+      <x:c r="B1" s="17"/>
+      <x:c r="C1" s="17"/>
+      <x:c r="D1" s="17"/>
+      <x:c r="E1" s="18"/>
+      <x:c r="F1" s="18"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="16" t="str">
+      <x:c r="A2" s="19" t="str">
         <x:v>schema_version</x:v>
       </x:c>
-      <x:c r="B2" s="16" t="str">
+      <x:c r="B2" s="19" t="str">
         <x:v>plan_id</x:v>
       </x:c>
-      <x:c r="C2" s="16" t="str">
+      <x:c r="C2" s="19" t="str">
         <x:v>plan_name</x:v>
       </x:c>
-      <x:c r="D2" s="16" t="str">
+      <x:c r="D2" s="19" t="str">
         <x:v>timezone</x:v>
       </x:c>
+      <x:c r="E2" s="18"/>
+      <x:c r="F2" s="18"/>
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
-      <x:c r="A3" s="17" t="n">
+      <x:c r="A3" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B3" s="17" t="str">
+      <x:c r="B3" s="20" t="str">
         <x:v>my-training</x:v>
       </x:c>
-      <x:c r="C3" s="17" t="str">
+      <x:c r="C3" s="20" t="str">
         <x:v>My training strategy</x:v>
       </x:c>
-      <x:c r="D3" s="17" t="str">
+      <x:c r="D3" s="20" t="str">
         <x:v>Europe/Berlin</x:v>
       </x:c>
+      <x:c r="E3" s="18"/>
+      <x:c r="F3" s="18"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="18"/>
       <x:c r="B4" s="18"/>
       <x:c r="C4" s="18"/>
       <x:c r="D4" s="18"/>
+      <x:c r="E4" s="18"/>
+      <x:c r="F4" s="18"/>
     </x:row>
     <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="15" t="str">
+      <x:c r="A5" s="17" t="str">
         <x:v>Goals</x:v>
       </x:c>
-      <x:c r="B5" s="15"/>
-      <x:c r="C5" s="15"/>
+      <x:c r="B5" s="17"/>
+      <x:c r="C5" s="17"/>
       <x:c r="D5" s="18"/>
+      <x:c r="E5" s="18"/>
+      <x:c r="F5" s="18"/>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
-      <x:c r="A6" s="16" t="str">
+      <x:c r="A6" s="19" t="str">
         <x:v>goal_id</x:v>
       </x:c>
-      <x:c r="B6" s="16" t="str">
+      <x:c r="B6" s="19" t="str">
         <x:v>title</x:v>
       </x:c>
-      <x:c r="C6" s="16" t="str">
+      <x:c r="C6" s="19" t="str">
         <x:v>benchmark</x:v>
       </x:c>
       <x:c r="D6" s="18"/>
+      <x:c r="E6" s="18"/>
+      <x:c r="F6" s="18"/>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
-      <x:c r="A7" s="17" t="str">
+      <x:c r="A7" s="20" t="str">
         <x:v>muscle-up</x:v>
       </x:c>
-      <x:c r="B7" s="17" t="str">
+      <x:c r="B7" s="20" t="str">
         <x:v>Muscle-up</x:v>
       </x:c>
-      <x:c r="C7" s="17" t="str">
+      <x:c r="C7" s="20" t="str">
         <x:v>1 unassisted repetition</x:v>
       </x:c>
       <x:c r="D7" s="18"/>
+      <x:c r="E7" s="18"/>
+      <x:c r="F7" s="18"/>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
-      <x:c r="A8" s="17" t="str">
+      <x:c r="A8" s="20" t="str">
         <x:v>hspu</x:v>
       </x:c>
-      <x:c r="B8" s="17" t="str">
+      <x:c r="B8" s="20" t="str">
         <x:v>Handstand push-up</x:v>
       </x:c>
-      <x:c r="C8" s="17" t="str">
+      <x:c r="C8" s="20" t="str">
         <x:v>1 controlled repetition</x:v>
       </x:c>
       <x:c r="D8" s="18"/>
+      <x:c r="E8" s="18"/>
+      <x:c r="F8" s="18"/>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
-      <x:c r="A9" s="17" t="str">
+      <x:c r="A9" s="20" t="str">
         <x:v>pistol</x:v>
       </x:c>
-      <x:c r="B9" s="17" t="str">
+      <x:c r="B9" s="20" t="str">
         <x:v>Pistol squat</x:v>
       </x:c>
-      <x:c r="C9" s="17" t="str">
+      <x:c r="C9" s="20" t="str">
         <x:v>1 repetition on each side</x:v>
       </x:c>
       <x:c r="D9" s="18"/>
+      <x:c r="E9" s="18"/>
+      <x:c r="F9" s="18"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="18"/>
       <x:c r="B10" s="18"/>
       <x:c r="C10" s="18"/>
       <x:c r="D10" s="18"/>
+      <x:c r="E10" s="18"/>
+      <x:c r="F10" s="18"/>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="15" t="str">
+      <x:c r="A11" s="17" t="str">
         <x:v>Parts</x:v>
       </x:c>
-      <x:c r="B11" s="15"/>
-      <x:c r="C11" s="15"/>
-      <x:c r="D11" s="15"/>
+      <x:c r="B11" s="17"/>
+      <x:c r="C11" s="17"/>
+      <x:c r="D11" s="17"/>
+      <x:c r="E11" s="18"/>
+      <x:c r="F11" s="18"/>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="16" t="str">
+      <x:c r="A12" s="19" t="str">
         <x:v>part_id</x:v>
       </x:c>
-      <x:c r="B12" s="16" t="str">
+      <x:c r="B12" s="19" t="str">
         <x:v>version</x:v>
       </x:c>
-      <x:c r="C12" s="16" t="str">
+      <x:c r="C12" s="19" t="str">
         <x:v>title</x:v>
       </x:c>
-      <x:c r="D12" s="16" t="str">
+      <x:c r="D12" s="19" t="str">
         <x:v>prescription</x:v>
       </x:c>
+      <x:c r="E12" s="18"/>
+      <x:c r="F12" s="18"/>
     </x:row>
     <x:row r="13" ht="64" customHeight="1">
-      <x:c r="A13" s="17" t="str">
+      <x:c r="A13" s="20" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="B13" s="17" t="str">
+      <x:c r="B13" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C13" s="17" t="str">
+      <x:c r="C13" s="20" t="str">
         <x:v>Skills A</x:v>
       </x:c>
-      <x:c r="D13" s="22" t="str">
+      <x:c r="D13" s="26" t="str">
         <x:v>Muscle-up + pistol practice, then Core circuit (5 rounds). Record variation, assistance, sets and reps.</x:v>
       </x:c>
+      <x:c r="E13" s="18"/>
+      <x:c r="F13" s="18"/>
     </x:row>
     <x:row r="14" ht="64" customHeight="1">
-      <x:c r="A14" s="17" t="str">
+      <x:c r="A14" s="20" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="B14" s="17" t="str">
+      <x:c r="B14" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C14" s="17" t="str">
+      <x:c r="C14" s="20" t="str">
         <x:v>Skills B</x:v>
       </x:c>
-      <x:c r="D14" s="22" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>Handstand push-up + pistol practice, then Core circuit (5 rounds). Record variation, assistance, sets and reps.</x:v>
       </x:c>
+      <x:c r="E14" s="18"/>
+      <x:c r="F14" s="18"/>
     </x:row>
     <x:row r="15" ht="26" customHeight="1">
-      <x:c r="A15" s="17" t="str">
+      <x:c r="A15" s="20" t="str">
         <x:v>Technique</x:v>
       </x:c>
-      <x:c r="B15" s="17" t="str">
+      <x:c r="B15" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C15" s="17" t="str">
+      <x:c r="C15" s="20" t="str">
         <x:v>Light technique</x:v>
       </x:c>
-      <x:c r="D15" s="22" t="str">
+      <x:c r="D15" s="26" t="str">
         <x:v>Easy handstand practice. Record the variation and hold time.</x:v>
       </x:c>
+      <x:c r="E15" s="18"/>
+      <x:c r="F15" s="18"/>
     </x:row>
     <x:row r="16" ht="96" customHeight="1">
-      <x:c r="A16" s="17" t="str">
+      <x:c r="A16" s="20" t="str">
         <x:v>Core</x:v>
       </x:c>
-      <x:c r="B16" s="17" t="str">
+      <x:c r="B16" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C16" s="17" t="str">
+      <x:c r="C16" s="20" t="str">
         <x:v>Core circuit — 16 min 40 sec</x:v>
       </x:c>
-      <x:c r="D16" s="22" t="str">
+      <x:c r="D16" s="26" t="str">
         <x:v>5 rounds: pull-ups, push-ups, weighted squats, upside-down hanging shoulder/ab work. Each exercise: 30 sec work + 20 sec rest, then continue around the circuit. 5 × 4 × 50 sec = 16 min 40 sec including the final rest.</x:v>
       </x:c>
+      <x:c r="E16" s="18"/>
+      <x:c r="F16" s="18"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="18"/>
       <x:c r="B17" s="18"/>
       <x:c r="C17" s="18"/>
       <x:c r="D17" s="18"/>
+      <x:c r="E17" s="18"/>
+      <x:c r="F17" s="18"/>
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
-      <x:c r="A18" s="15" t="str">
+      <x:c r="A18" s="17" t="str">
         <x:v>PartGoals</x:v>
       </x:c>
-      <x:c r="B18" s="15"/>
-      <x:c r="C18" s="15"/>
+      <x:c r="B18" s="17"/>
+      <x:c r="C18" s="17"/>
       <x:c r="D18" s="18"/>
+      <x:c r="E18" s="18"/>
+      <x:c r="F18" s="18"/>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
-      <x:c r="A19" s="16" t="str">
+      <x:c r="A19" s="19" t="str">
         <x:v>part_id</x:v>
       </x:c>
-      <x:c r="B19" s="16" t="str">
+      <x:c r="B19" s="19" t="str">
         <x:v>version</x:v>
       </x:c>
-      <x:c r="C19" s="16" t="str">
+      <x:c r="C19" s="19" t="str">
         <x:v>goal_id</x:v>
       </x:c>
       <x:c r="D19" s="18"/>
+      <x:c r="E19" s="18"/>
+      <x:c r="F19" s="18"/>
     </x:row>
     <x:row r="20" ht="26" customHeight="1">
-      <x:c r="A20" s="17" t="str">
+      <x:c r="A20" s="20" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="B20" s="17" t="str">
+      <x:c r="B20" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C20" s="17" t="str">
+      <x:c r="C20" s="20" t="str">
         <x:v>muscle-up</x:v>
       </x:c>
       <x:c r="D20" s="18"/>
+      <x:c r="E20" s="18"/>
+      <x:c r="F20" s="18"/>
     </x:row>
     <x:row r="21" ht="26" customHeight="1">
-      <x:c r="A21" s="17" t="str">
+      <x:c r="A21" s="20" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="B21" s="17" t="str">
+      <x:c r="B21" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C21" s="17" t="str">
+      <x:c r="C21" s="20" t="str">
         <x:v>pistol</x:v>
       </x:c>
       <x:c r="D21" s="18"/>
+      <x:c r="E21" s="18"/>
+      <x:c r="F21" s="18"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
-      <x:c r="A22" s="17" t="str">
+      <x:c r="A22" s="20" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="B22" s="17" t="str">
+      <x:c r="B22" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C22" s="17" t="str">
+      <x:c r="C22" s="20" t="str">
         <x:v>hspu</x:v>
       </x:c>
       <x:c r="D22" s="18"/>
+      <x:c r="E22" s="18"/>
+      <x:c r="F22" s="18"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
-      <x:c r="A23" s="17" t="str">
+      <x:c r="A23" s="20" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="B23" s="17" t="str">
+      <x:c r="B23" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C23" s="17" t="str">
+      <x:c r="C23" s="20" t="str">
         <x:v>pistol</x:v>
       </x:c>
       <x:c r="D23" s="18"/>
+      <x:c r="E23" s="18"/>
+      <x:c r="F23" s="18"/>
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
-      <x:c r="A24" s="17" t="str">
+      <x:c r="A24" s="20" t="str">
         <x:v>Technique</x:v>
       </x:c>
-      <x:c r="B24" s="17" t="str">
+      <x:c r="B24" s="20" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C24" s="17" t="str">
+      <x:c r="C24" s="20" t="str">
         <x:v>hspu</x:v>
       </x:c>
       <x:c r="D24" s="18"/>
+      <x:c r="E24" s="18"/>
+      <x:c r="F24" s="18"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="18"/>
+      <x:c r="B25" s="18"/>
+      <x:c r="C25" s="18"/>
+      <x:c r="D25" s="18"/>
+      <x:c r="E25" s="18"/>
+      <x:c r="F25" s="18"/>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="A26" s="17" t="str">
+        <x:v>Weekly schedule</x:v>
+      </x:c>
+      <x:c r="B26" s="17"/>
+      <x:c r="C26" s="17"/>
+      <x:c r="D26" s="17"/>
+      <x:c r="E26" s="17"/>
+      <x:c r="F26" s="17"/>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="A27" s="19" t="str">
+        <x:v>Day</x:v>
+      </x:c>
+      <x:c r="B27" s="19" t="str">
+        <x:v>Time</x:v>
+      </x:c>
+      <x:c r="C27" s="19" t="str">
+        <x:v>Minutes</x:v>
+      </x:c>
+      <x:c r="D27" s="19" t="str">
+        <x:v>Activity</x:v>
+      </x:c>
+      <x:c r="E27" s="19" t="str">
+        <x:v>Recorded by</x:v>
+      </x:c>
+      <x:c r="F27" s="19" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="26" customHeight="1">
+      <x:c r="A28" s="20" t="str">
+        <x:v>Monday</x:v>
+      </x:c>
+      <x:c r="B28" s="21"/>
+      <x:c r="C28" s="22"/>
+      <x:c r="D28" s="20"/>
+      <x:c r="E28" s="20"/>
+      <x:c r="F28" s="20"/>
+    </x:row>
+    <x:row r="29" ht="26" customHeight="1">
+      <x:c r="A29" s="20" t="str">
+        <x:v>Tuesday</x:v>
+      </x:c>
+      <x:c r="B29" s="21"/>
+      <x:c r="C29" s="22"/>
+      <x:c r="D29" s="20"/>
+      <x:c r="E29" s="20"/>
+      <x:c r="F29" s="20"/>
+    </x:row>
+    <x:row r="30" ht="26" customHeight="1">
+      <x:c r="A30" s="20" t="str">
+        <x:v>Wednesday</x:v>
+      </x:c>
+      <x:c r="B30" s="21"/>
+      <x:c r="C30" s="22"/>
+      <x:c r="D30" s="20"/>
+      <x:c r="E30" s="20"/>
+      <x:c r="F30" s="20"/>
+    </x:row>
+    <x:row r="31" ht="26" customHeight="1">
+      <x:c r="A31" s="20" t="str">
+        <x:v>Thursday</x:v>
+      </x:c>
+      <x:c r="B31" s="21"/>
+      <x:c r="C31" s="22"/>
+      <x:c r="D31" s="20"/>
+      <x:c r="E31" s="20"/>
+      <x:c r="F31" s="20"/>
+    </x:row>
+    <x:row r="32" ht="26" customHeight="1">
+      <x:c r="A32" s="20" t="str">
+        <x:v>Friday</x:v>
+      </x:c>
+      <x:c r="B32" s="21"/>
+      <x:c r="C32" s="22"/>
+      <x:c r="D32" s="20"/>
+      <x:c r="E32" s="20"/>
+      <x:c r="F32" s="20"/>
+    </x:row>
+    <x:row r="33" ht="26" customHeight="1">
+      <x:c r="A33" s="20" t="str">
+        <x:v>Saturday</x:v>
+      </x:c>
+      <x:c r="B33" s="21"/>
+      <x:c r="C33" s="22"/>
+      <x:c r="D33" s="20"/>
+      <x:c r="E33" s="20"/>
+      <x:c r="F33" s="20"/>
+    </x:row>
+    <x:row r="34" ht="26" customHeight="1">
+      <x:c r="A34" s="20" t="str">
+        <x:v>Sunday</x:v>
+      </x:c>
+      <x:c r="B34" s="21"/>
+      <x:c r="C34" s="22"/>
+      <x:c r="D34" s="20"/>
+      <x:c r="E34" s="20"/>
+      <x:c r="F34" s="20"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="E28:E100">
+      <x:formula1>"Garmin,Other tracker,No manual log"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -687,156 +860,156 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="16" t="str">
+      <x:c r="A1" s="19" t="str">
         <x:v>Date</x:v>
       </x:c>
-      <x:c r="B1" s="16" t="str">
+      <x:c r="B1" s="19" t="str">
         <x:v>Block</x:v>
       </x:c>
-      <x:c r="C1" s="16" t="str">
+      <x:c r="C1" s="19" t="str">
         <x:v>Plan</x:v>
       </x:c>
-      <x:c r="D1" s="16" t="str">
+      <x:c r="D1" s="19" t="str">
         <x:v>Core done</x:v>
       </x:c>
-      <x:c r="E1" s="16" t="str">
+      <x:c r="E1" s="19" t="str">
         <x:v>Muscle-up result</x:v>
       </x:c>
-      <x:c r="F1" s="16" t="str">
+      <x:c r="F1" s="19" t="str">
         <x:v>HSPU result</x:v>
       </x:c>
-      <x:c r="G1" s="16" t="str">
+      <x:c r="G1" s="19" t="str">
         <x:v>Pistol result</x:v>
       </x:c>
-      <x:c r="H1" s="16" t="str">
+      <x:c r="H1" s="19" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="24" t="d">
+      <x:c r="A2" s="28" t="d">
         <x:v>2026-10-19T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="B2" s="20" t="str">
+      <x:c r="B2" s="24" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="C2" s="23" t="str">
+      <x:c r="C2" s="27" t="str">
         <x:v>Muscle-up + pistol practice, then core circuit</x:v>
       </x:c>
-      <x:c r="D2" s="21" t="b">
+      <x:c r="D2" s="25" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E2" s="17"/>
-      <x:c r="F2" s="17"/>
-      <x:c r="G2" s="17"/>
-      <x:c r="H2" s="17"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
+      <x:c r="H2" s="20"/>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
-      <x:c r="A3" s="24" t="d">
+      <x:c r="A3" s="28" t="d">
         <x:v>2026-10-20T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="B3" s="20" t="str">
+      <x:c r="B3" s="24" t="str">
         <x:v>Technique</x:v>
       </x:c>
-      <x:c r="C3" s="23" t="str">
+      <x:c r="C3" s="27" t="str">
         <x:v>Light handstand technique</x:v>
       </x:c>
-      <x:c r="D3" s="21" t="b">
+      <x:c r="D3" s="25" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E3" s="17"/>
-      <x:c r="F3" s="17"/>
-      <x:c r="G3" s="17"/>
-      <x:c r="H3" s="17"/>
+      <x:c r="E3" s="20"/>
+      <x:c r="F3" s="20"/>
+      <x:c r="G3" s="20"/>
+      <x:c r="H3" s="20"/>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
-      <x:c r="A4" s="24" t="d">
+      <x:c r="A4" s="28" t="d">
         <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="B4" s="20" t="str">
+      <x:c r="B4" s="24" t="str">
         <x:v>Empty</x:v>
       </x:c>
-      <x:c r="C4" s="23" t="str">
+      <x:c r="C4" s="27" t="str">
         <x:v>Rest or other sport</x:v>
       </x:c>
-      <x:c r="D4" s="21" t="b">
+      <x:c r="D4" s="25" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E4" s="17"/>
-      <x:c r="F4" s="17"/>
-      <x:c r="G4" s="17"/>
-      <x:c r="H4" s="17"/>
+      <x:c r="E4" s="20"/>
+      <x:c r="F4" s="20"/>
+      <x:c r="G4" s="20"/>
+      <x:c r="H4" s="20"/>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="24" t="d">
+      <x:c r="A5" s="28" t="d">
         <x:v>2026-10-22T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="B5" s="20" t="str">
+      <x:c r="B5" s="24" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C5" s="23" t="str">
+      <x:c r="C5" s="27" t="str">
         <x:v>Handstand push-up + pistol practice, then core circuit</x:v>
       </x:c>
-      <x:c r="D5" s="21" t="b">
+      <x:c r="D5" s="25" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E5" s="17"/>
-      <x:c r="F5" s="17"/>
-      <x:c r="G5" s="17"/>
-      <x:c r="H5" s="17"/>
+      <x:c r="E5" s="20"/>
+      <x:c r="F5" s="20"/>
+      <x:c r="G5" s="20"/>
+      <x:c r="H5" s="20"/>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
-      <x:c r="A6" s="24" t="d">
+      <x:c r="A6" s="28" t="d">
         <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="B6" s="20" t="str">
+      <x:c r="B6" s="24" t="str">
         <x:v>Empty</x:v>
       </x:c>
-      <x:c r="C6" s="23" t="str">
+      <x:c r="C6" s="27" t="str">
         <x:v>Rest or other sport</x:v>
       </x:c>
-      <x:c r="D6" s="21" t="b">
+      <x:c r="D6" s="25" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E6" s="17"/>
-      <x:c r="F6" s="17"/>
-      <x:c r="G6" s="17"/>
-      <x:c r="H6" s="17"/>
+      <x:c r="E6" s="20"/>
+      <x:c r="F6" s="20"/>
+      <x:c r="G6" s="20"/>
+      <x:c r="H6" s="20"/>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
-      <x:c r="A7" s="24" t="d">
+      <x:c r="A7" s="28" t="d">
         <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="B7" s="20" t="str">
+      <x:c r="B7" s="24" t="str">
         <x:v>Technique</x:v>
       </x:c>
-      <x:c r="C7" s="23" t="str">
+      <x:c r="C7" s="27" t="str">
         <x:v>Light skill practice</x:v>
       </x:c>
-      <x:c r="D7" s="21" t="b">
+      <x:c r="D7" s="25" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E7" s="17"/>
-      <x:c r="F7" s="17"/>
-      <x:c r="G7" s="17"/>
-      <x:c r="H7" s="17"/>
+      <x:c r="E7" s="20"/>
+      <x:c r="F7" s="20"/>
+      <x:c r="G7" s="20"/>
+      <x:c r="H7" s="20"/>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
-      <x:c r="A8" s="24" t="d">
+      <x:c r="A8" s="28" t="d">
         <x:v>2026-10-25T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="B8" s="20" t="str">
+      <x:c r="B8" s="24" t="str">
         <x:v>Empty</x:v>
       </x:c>
-      <x:c r="C8" s="23" t="str">
+      <x:c r="C8" s="27" t="str">
         <x:v>Rest or other sport</x:v>
       </x:c>
-      <x:c r="D8" s="21" t="b">
+      <x:c r="D8" s="25" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E8" s="17"/>
-      <x:c r="F8" s="17"/>
-      <x:c r="G8" s="17"/>
-      <x:c r="H8" s="17"/>
+      <x:c r="E8" s="20"/>
+      <x:c r="F8" s="20"/>
+      <x:c r="G8" s="20"/>
+      <x:c r="H8" s="20"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">

</xml_diff>